<commit_message>
Prepare automation-billing repository with current project files
</commit_message>
<xml_diff>
--- a/dummy_attendance_records.xlsx
+++ b/dummy_attendance_records.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance_Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,9 +16,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +27,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FFffffff"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -41,12 +48,33 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000008B"/>
-        <bgColor rgb="0000008B"/>
+        <fgColor rgb="FF00008b"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFc6c6c6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFc6c6c6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFc6c6c6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFc6c6c6"/>
+      </bottom>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -56,15 +84,31 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -143,10 +187,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -184,69 +228,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -270,54 +316,53 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -327,7 +372,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -336,7 +381,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -345,7 +390,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -353,10 +398,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -385,7 +430,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -398,13 +443,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -424,26 +468,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="12.005" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="15.005" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
+    <col width="16.005" bestFit="1" customWidth="1" style="5" min="3" max="3"/>
+    <col width="19.005" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="15.005" bestFit="1" customWidth="1" style="5" min="5" max="5"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="6" min="6" max="6"/>
+    <col width="17.005" bestFit="1" customWidth="1" style="6" min="7" max="7"/>
+    <col width="21.005" bestFit="1" customWidth="1" style="6" min="8" max="8"/>
+    <col width="10.005" bestFit="1" customWidth="1" style="5" min="9" max="9"/>
+    <col width="21.005" bestFit="1" customWidth="1" style="5" min="10" max="10"/>
+    <col width="26.005" bestFit="1" customWidth="1" style="5" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>period_key</t>
@@ -469,17 +513,17 @@
           <t>location_code</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>days_worked</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>approved_leaves</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>unapproved_absences</t>
         </is>
@@ -500,313 +544,309 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="19.5" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>EMP-1001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Alice Smith</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>alice@axian.com</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>workwithzain09@gmail.com</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>US-MAIN</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
+      <c r="K2" s="5" t="n"/>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="19.5" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>EMP-1002</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Bob Jones</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>bob@axian.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>241896@students.au.edu.pk</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>US-MAIN</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>Sick leave approved</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="19.5" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>EMP-1004</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Diana Prince</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>diana@axian.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>zainkhantge2@gmail.com</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>US-MAIN</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Missed some days</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="19.5" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>EMP-1003</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Charlie Brown</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>charlie@axian.com</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>beattlerokkie17679@gmail.com</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>US-MAIN</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>No call no show</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>EMP-1005</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Eve Adams</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>eve@axian.com</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>workwithzain02@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>US-MAIN</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>INACTIVE</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Was terminated mid-month</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="19.5" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>EMP-9999</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Ghost Employee</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>ghost@axian.com</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>US-MAIN</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>INACTIVE</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Was terminated mid-month</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>EMP-9999</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Ghost Employee</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ghost@axian.com</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>US-MAIN</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Not in master DB</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="J2:J7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PENDING,VERIFIED,DISCREPANCY_FLAGGED"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>